<commit_message>
[EDP-DDM-31133] Updated platform system requirements, guide and calculator: master -> 3 x r5.2xlarge; worker -> 3 x r5.2xlarge.
Change-Id: Icc0a064c250cdbbc95e17cd07871b13d7c61eb07
</commit_message>
<xml_diff>
--- a/docs/en/modules/arch/attachments/architecture/platform-system-requirements/registry-cost-calculator.xlsx
+++ b/docs/en/modules/arch/attachments/architecture/platform-system-requirements/registry-cost-calculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Anton_Tuhai\Documents\Gerrit\test\ddm-architecture\docs\en\modules\arch\attachments\architecture\platform-system-requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Maksym_Kharchenko/Work/Development/mdtu-ddm/mdtu-ddm-gerrit-workspace/mdtu-ddm/general/ddm-architecture/docs/en/modules/arch/attachments/architecture/platform-system-requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0E1DEF-1CC3-4A82-BA9B-F9E6980C862A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888034B4-566D-184C-B96B-11934D53822C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{27F18D04-7E62-4946-83A8-E11013D50C84}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="17640" xr2:uid="{27F18D04-7E62-4946-83A8-E11013D50C84}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost calculator" sheetId="1" r:id="rId1"/>
@@ -365,7 +365,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -610,7 +610,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -626,9 +626,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Офіс">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -666,7 +666,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Офіс">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -772,7 +772,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Офіс">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -914,7 +914,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -923,31 +923,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2669E3AB-101C-8547-83F4-DF3AE92242F5}">
   <dimension ref="A1:V24"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.125" customWidth="1"/>
+    <col min="1" max="1" width="25.1640625" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.125" customWidth="1"/>
-    <col min="4" max="4" width="11.875" customWidth="1"/>
-    <col min="5" max="5" width="8.625" customWidth="1"/>
-    <col min="6" max="6" width="9.125" customWidth="1"/>
-    <col min="7" max="7" width="10.125" customWidth="1"/>
-    <col min="8" max="8" width="10.625" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" customWidth="1"/>
+    <col min="4" max="4" width="11.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="9.1640625" customWidth="1"/>
+    <col min="7" max="7" width="10.1640625" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" customWidth="1"/>
     <col min="9" max="9" width="11.5" customWidth="1"/>
-    <col min="10" max="10" width="11.875" customWidth="1"/>
-    <col min="11" max="11" width="8.625" customWidth="1"/>
+    <col min="10" max="10" width="11.83203125" customWidth="1"/>
+    <col min="11" max="11" width="8.6640625" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
     <col min="13" max="13" width="11.5" customWidth="1"/>
-    <col min="14" max="18" width="12.125" customWidth="1"/>
-    <col min="20" max="20" width="13.125" customWidth="1"/>
+    <col min="14" max="18" width="12.1640625" customWidth="1"/>
+    <col min="20" max="20" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" s="8"/>
       <c r="C1" s="28"/>
       <c r="D1" s="28"/>
     </row>
-    <row r="2" spans="1:22">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -958,7 +958,7 @@
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
     </row>
-    <row r="3" spans="1:22">
+    <row r="3" spans="1:22" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
@@ -974,7 +974,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:22">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
         <v>4</v>
       </c>
@@ -984,7 +984,7 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" s="29" t="s">
         <v>5</v>
       </c>
@@ -1010,7 +1010,7 @@
       <c r="U6" s="29"/>
       <c r="V6" s="29"/>
     </row>
-    <row r="7" spans="1:22" ht="80.25" customHeight="1">
+    <row r="7" spans="1:22" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:22" ht="18" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>28</v>
       </c>
@@ -1150,14 +1150,14 @@
       </c>
       <c r="U8" s="27">
         <f>J$24/$B$4*C8</f>
-        <v>129.26185000000001</v>
+        <v>116.83035</v>
       </c>
       <c r="V8" s="15">
         <f>T8+U8</f>
-        <v>319.62585000000001</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22">
+        <v>307.19434999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="18" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>31</v>
       </c>
@@ -1229,14 +1229,14 @@
       </c>
       <c r="U9" s="27">
         <f>J$24/$B$4*C9</f>
-        <v>258.52370000000002</v>
+        <v>233.66069999999999</v>
       </c>
       <c r="V9" s="15">
         <f>T9+U9</f>
-        <v>570.71170000000006</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22">
+        <v>545.84870000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
         <v>32</v>
       </c>
@@ -1308,14 +1308,14 @@
       </c>
       <c r="U10" s="27">
         <f>J$24/$B$4*C10</f>
-        <v>646.30925000000002</v>
+        <v>584.15174999999999</v>
       </c>
       <c r="V10" s="15">
         <f t="shared" ref="V10:V11" si="0">T10+U10</f>
-        <v>1323.9692500000001</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22">
+        <v>1261.8117500000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="18" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>33</v>
       </c>
@@ -1387,14 +1387,14 @@
       </c>
       <c r="U11" s="27">
         <f t="shared" ref="U11" si="2">J$24/$B$4*C11</f>
-        <v>1292.6185</v>
+        <v>1168.3035</v>
       </c>
       <c r="V11" s="15">
         <f t="shared" si="0"/>
-        <v>2579.3985000000002</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22">
+        <v>2455.0835000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" s="30" t="s">
         <v>34</v>
       </c>
@@ -1408,7 +1408,7 @@
       <c r="I15" s="30"/>
       <c r="J15" s="30"/>
     </row>
-    <row r="16" spans="1:22" ht="94.5">
+    <row r="16" spans="1:22" ht="85" x14ac:dyDescent="0.2">
       <c r="A16" s="13" t="s">
         <v>105</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>36</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>1356.12</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>39</v>
       </c>
@@ -1511,7 +1511,7 @@
         <v>2960.712</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>41</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>1134.9720000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>42</v>
       </c>
@@ -1555,14 +1555,14 @@
         <v>37</v>
       </c>
       <c r="C20" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D20" s="3">
         <v>0.60799999999999998</v>
       </c>
       <c r="E20" s="3">
         <f t="shared" si="3"/>
-        <v>3.04</v>
+        <v>1.8239999999999998</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>38</v>
@@ -1576,14 +1576,14 @@
       </c>
       <c r="I20" s="3">
         <f t="shared" si="4"/>
-        <v>148.75</v>
+        <v>89.25</v>
       </c>
       <c r="J20" s="3">
         <f t="shared" si="5"/>
-        <v>2337.5500000000002</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" s="21" customFormat="1">
+        <v>1402.53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" s="21" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="20" t="s">
         <v>43</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>456.8</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="21" customFormat="1">
+    <row r="22" spans="1:10" s="21" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="20" t="s">
         <v>44</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>685.28</v>
       </c>
     </row>
-    <row r="23" spans="1:10" s="21" customFormat="1">
+    <row r="23" spans="1:10" s="21" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="20" t="s">
         <v>45</v>
       </c>
@@ -1688,13 +1688,13 @@
         <v>456.8</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="I24" s="16" t="s">
         <v>46</v>
       </c>
       <c r="J24" s="15">
         <f>SUM(J17:J23)+SUM(I17:I23)</f>
-        <v>10340.948</v>
+        <v>9346.4279999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1712,15 +1712,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A819B9D-8FE0-401F-8C51-9F6F8ACD5799}">
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="49.625" customWidth="1"/>
-    <col min="2" max="3" width="15.125" customWidth="1"/>
-    <col min="4" max="4" width="14.625" customWidth="1"/>
-    <col min="6" max="6" width="12.625" customWidth="1"/>
+    <col min="1" max="1" width="49.6640625" customWidth="1"/>
+    <col min="2" max="3" width="15.1640625" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1" s="22" t="s">
         <v>8</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -1738,13 +1738,13 @@
       </c>
       <c r="C2">
         <f>B2*C6*720*'Cost calculator'!E8+B2*'Cost calculator'!I8+'Cost calculator'!M8+'Cost calculator'!S8+B2*'Cost calculator'!U8</f>
-        <v>570.71170000000006</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>545.84870000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F3" s="21"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="22" t="s">
         <v>49</v>
       </c>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="F4" s="21"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="str">
         <f>Glossary!A1</f>
         <v>High availability</v>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="F5" s="21"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="str">
         <f>Glossary!C1</f>
         <v>Operating mode</v>
@@ -1780,7 +1780,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="22" t="s">
         <v>106</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
         <f>Glossary!A6</f>
         <v>Number of business entities</v>
@@ -1801,7 +1801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <f>Glossary!C6</f>
         <v>Maximum number of instances of business entities (rows in a table)</v>
@@ -1814,7 +1814,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="str">
         <f>Glossary!E6</f>
         <v>Approximate volume of historical data in GB</v>
@@ -1827,7 +1827,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="22" t="s">
         <v>57</v>
       </c>
@@ -1850,7 +1850,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="str">
         <f>Glossary!A12</f>
         <v>Number of users</v>
@@ -1877,7 +1877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="str">
         <f>Glossary!C12</f>
         <v>Number of services (business processes)</v>
@@ -1904,7 +1904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="str">
         <f>Glossary!E12</f>
         <v>Average number of user tasks per service</v>
@@ -1926,7 +1926,7 @@
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
     </row>
-    <row r="20" spans="1:7">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="str">
         <f>Glossary!G12</f>
         <v>Average number of automated tasks per service</v>
@@ -1953,7 +1953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="str">
         <f>Glossary!I12</f>
         <v>Number of reports</v>
@@ -1970,7 +1970,7 @@
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
     </row>
-    <row r="22" spans="1:7">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="str">
         <f>Glossary!K12</f>
         <v>Number of excerpts</v>
@@ -1997,7 +1997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="str">
         <f>Glossary!M12</f>
         <v>Number of services provided per month</v>
@@ -2019,7 +2019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="21"/>
       <c r="C24">
         <f>MAX(C17:C23)</f>
@@ -2199,19 +2199,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7C2CE02-549B-42BB-BB2B-79BD8E0A657F}">
   <dimension ref="A1:N27"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.625" customWidth="1"/>
-    <col min="2" max="2" width="15.875" customWidth="1"/>
-    <col min="3" max="3" width="42.875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="42.625" customWidth="1"/>
-    <col min="7" max="7" width="44.125" customWidth="1"/>
-    <col min="9" max="9" width="15.625" customWidth="1"/>
-    <col min="11" max="11" width="23.875" customWidth="1"/>
-    <col min="13" max="13" width="39.625" customWidth="1"/>
+    <col min="1" max="1" width="27.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="42.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.6640625" customWidth="1"/>
+    <col min="7" max="7" width="44.1640625" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="11" max="11" width="23.83203125" customWidth="1"/>
+    <col min="13" max="13" width="39.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="22" t="s">
         <v>68</v>
       </c>
@@ -2225,7 +2225,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>70</v>
       </c>
@@ -2239,7 +2239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C4" t="s">
         <v>72</v>
       </c>
@@ -2262,7 +2262,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
         <v>73</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>54</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="24" t="s">
         <v>76</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>79</v>
       </c>
@@ -2342,12 +2342,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="22" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="22" t="s">
         <v>82</v>
       </c>
@@ -2391,7 +2391,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>61</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="24" t="s">
         <v>89</v>
       </c>
@@ -2467,7 +2467,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>92</v>
       </c>
@@ -2505,12 +2505,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="22" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="22" t="s">
         <v>82</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -2592,7 +2592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="24" t="s">
         <v>94</v>
       </c>
@@ -2631,7 +2631,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>97</v>
       </c>
@@ -2669,12 +2669,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="22" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="22" t="s">
         <v>82</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>63</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="24" t="s">
         <v>100</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>103</v>
       </c>
@@ -2840,28 +2840,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="346a80a9-3278-4844-b436-58ae57568790">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="a2d094e0-efa8-4820-a0b3-29af30f3c512" xsi:nil="true"/>
-    <SharedWithUsers xmlns="a2d094e0-efa8-4820-a0b3-29af30f3c512">
-      <UserInfo>
-        <DisplayName>Vitalii Fedorenko</DisplayName>
-        <AccountId>158</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Oleksandr Zakusylo</DisplayName>
-        <AccountId>159</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <Capability_x0020_name xmlns="346a80a9-3278-4844-b436-58ae57568790"/>
-    <Release xmlns="346a80a9-3278-4844-b436-58ae57568790" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3124,21 +3108,34 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="346a80a9-3278-4844-b436-58ae57568790">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a2d094e0-efa8-4820-a0b3-29af30f3c512" xsi:nil="true"/>
+    <SharedWithUsers xmlns="a2d094e0-efa8-4820-a0b3-29af30f3c512">
+      <UserInfo>
+        <DisplayName>Vitalii Fedorenko</DisplayName>
+        <AccountId>158</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Oleksandr Zakusylo</DisplayName>
+        <AccountId>159</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <Capability_x0020_name xmlns="346a80a9-3278-4844-b436-58ae57568790"/>
+    <Release xmlns="346a80a9-3278-4844-b436-58ae57568790" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD363066-8CBD-4D6F-8835-7EB8A1E12EC9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92FEC7CF-4815-42BA-A053-9D2F9AB7FD60}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="346a80a9-3278-4844-b436-58ae57568790"/>
-    <ds:schemaRef ds:uri="a2d094e0-efa8-4820-a0b3-29af30f3c512"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3163,9 +3160,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92FEC7CF-4815-42BA-A053-9D2F9AB7FD60}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD363066-8CBD-4D6F-8835-7EB8A1E12EC9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="346a80a9-3278-4844-b436-58ae57568790"/>
+    <ds:schemaRef ds:uri="a2d094e0-efa8-4820-a0b3-29af30f3c512"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>